<commit_message>
docs: freeze Sprint 0 async import contract
</commit_message>
<xml_diff>
--- a/deliverables/pm/excel_templates/01_products_v1.0.xlsx
+++ b/deliverables/pm/excel_templates/01_products_v1.0.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入模板" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="正确样例" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误样例" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举值" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入模板" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="正确样例" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误样例" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举值" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'导入模板'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'正确样例'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'错误样例'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'枚举值'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导入模板'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'正确样例'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'错误样例'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'枚举值'!$A$1:$A$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -626,6 +627,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>schemaIdentifier</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>jiugeng.amazon.erp.import</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>importType</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>templateVersion</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>maxDataRows</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -693,7 +754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -803,7 +864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -996,7 +1057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>